<commit_message>
feat: Add excel spreadsheet import with user creation and email verification handling
</commit_message>
<xml_diff>
--- a/static/planilha_torneio.xlsx
+++ b/static/planilha_torneio.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Atletas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001a1a2e"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,120 +413,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Nome do Atleta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
-          <t>Cabeca de Chave</t>
+          <t>E-mail</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
-          <t>Carlos Silva</t>
+          <t>Verificado</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
-          <t>Categoria A</t>
+          <t>Cabeça de Chave</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Fernando Costa</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Categoria A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Roberto Lima</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Categoria A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Paulo Souza</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Categoria A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ana Paula</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Categoria B</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Maria José</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Categoria B</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>